<commit_message>
Wire real Submit button and feedback copy from translations
Uses the now-added quiz.submit_button_default and feedback.correct/
wrong.1-5 keys instead of the hardcoded English placeholders flagged
in the previous step. Verified with Playwright against both /en and
/es: correct default button label and correctly localized random
feedback text on answer submission.
</commit_message>
<xml_diff>
--- a/project-docs/quiz-translations-EN-ES.xlsx
+++ b/project-docs/quiz-translations-EN-ES.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2484,6 +2484,211 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" s="4" t="inlineStr">
+        <is>
+          <t>Quiz Question — Submit Button (default state)</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="n"/>
+      <c r="C131" s="5" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="6" t="inlineStr">
+        <is>
+          <t>quiz.submit_button_default</t>
+        </is>
+      </c>
+      <c r="B132" s="7" t="inlineStr">
+        <is>
+          <t>Submit</t>
+        </is>
+      </c>
+      <c r="C132" s="8" t="inlineStr">
+        <is>
+          <t>Enviar</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>Answer Feedback Messages (shown on the Submit button after answering)</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="n"/>
+      <c r="C133" s="5" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="6" t="inlineStr">
+        <is>
+          <t>feedback.correct.1</t>
+        </is>
+      </c>
+      <c r="B134" s="7" t="inlineStr">
+        <is>
+          <t>Correct! 🥳</t>
+        </is>
+      </c>
+      <c r="C134" s="8" t="inlineStr">
+        <is>
+          <t>¡Correcto! 🥳</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="6" t="inlineStr">
+        <is>
+          <t>feedback.correct.2</t>
+        </is>
+      </c>
+      <c r="B135" s="7" t="inlineStr">
+        <is>
+          <t>Just wow! 👏</t>
+        </is>
+      </c>
+      <c r="C135" s="8" t="inlineStr">
+        <is>
+          <t>¡Vaya! 👏</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="6" t="inlineStr">
+        <is>
+          <t>feedback.correct.3</t>
+        </is>
+      </c>
+      <c r="B136" s="7" t="inlineStr">
+        <is>
+          <t>Amazing! 🤩</t>
+        </is>
+      </c>
+      <c r="C136" s="8" t="inlineStr">
+        <is>
+          <t>¡Increíble! 🤩</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="6" t="inlineStr">
+        <is>
+          <t>feedback.correct.4</t>
+        </is>
+      </c>
+      <c r="B137" s="7" t="inlineStr">
+        <is>
+          <t>Nailed it! 💅</t>
+        </is>
+      </c>
+      <c r="C137" s="8" t="inlineStr">
+        <is>
+          <t>¡Acertaste! 💅</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="6" t="inlineStr">
+        <is>
+          <t>feedback.correct.5</t>
+        </is>
+      </c>
+      <c r="B138" s="7" t="inlineStr">
+        <is>
+          <t>You are on fire! 💃</t>
+        </is>
+      </c>
+      <c r="C138" s="8" t="inlineStr">
+        <is>
+          <t>¡Estás que ardes! 💃</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="6" t="inlineStr">
+        <is>
+          <t>feedback.wrong.1</t>
+        </is>
+      </c>
+      <c r="B139" s="7" t="inlineStr">
+        <is>
+          <t>Now you know... 🤷🏻‍♀️</t>
+        </is>
+      </c>
+      <c r="C139" s="8" t="inlineStr">
+        <is>
+          <t>Ahora ya lo sabes... 🤷🏻‍♀️</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="6" t="inlineStr">
+        <is>
+          <t>feedback.wrong.2</t>
+        </is>
+      </c>
+      <c r="B140" s="7" t="inlineStr">
+        <is>
+          <t>So close! 👀</t>
+        </is>
+      </c>
+      <c r="C140" s="8" t="inlineStr">
+        <is>
+          <t>¡Tan cerca! 👀</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="6" t="inlineStr">
+        <is>
+          <t>feedback.wrong.3</t>
+        </is>
+      </c>
+      <c r="B141" s="7" t="inlineStr">
+        <is>
+          <t>We're always learning 🧐</t>
+        </is>
+      </c>
+      <c r="C141" s="8" t="inlineStr">
+        <is>
+          <t>Siempre se aprende 🧐</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="6" t="inlineStr">
+        <is>
+          <t>feedback.wrong.4</t>
+        </is>
+      </c>
+      <c r="B142" s="7" t="inlineStr">
+        <is>
+          <t>Hmmm 🤔</t>
+        </is>
+      </c>
+      <c r="C142" s="8" t="inlineStr">
+        <is>
+          <t>Hmmm 🤔</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="6" t="inlineStr">
+        <is>
+          <t>feedback.wrong.5</t>
+        </is>
+      </c>
+      <c r="B143" s="7" t="inlineStr">
+        <is>
+          <t>Oops 🙈</t>
+        </is>
+      </c>
+      <c r="C143" s="8" t="inlineStr">
+        <is>
+          <t>Ups 🙈</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Wire finish.button_loading into the Check Result button's loading state
New translation key (EN: "Loading..." / ES: "Cargando...") swaps in for
finish.button while the submission request is in flight, replacing the
unlabeled disabled-only treatment used since step 9. Button stays
disabled during submission as before; only the label changes.

Verified against an artificially slow (2.5s) mock submission endpoint,
since the real one usually resolves too fast to reliably observe: both
locales show the correct loading label ("Loading..." / "Cargando...")
with the button disabled during the in-flight window, then proceed to
/result normally once the request resolves. Re-ran the standard full
regression against the real Apps Script deployment afterward to confirm
the real (fast) path still works end-to-end.
</commit_message>
<xml_diff>
--- a/project-docs/quiz-translations-EN-ES.xlsx
+++ b/project-docs/quiz-translations-EN-ES.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -963,1727 +963,1744 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
+          <t>finish.button_loading</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Loading...</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Cargando...</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
           <t>finish.policy</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>We highly value your privacy; therefore, please be informed that the Controller of data is SIA "Dynatech". Your personal data will be used only to organize the World Tourism Day Quiz and will be stored for a period of 30 days.</t>
         </is>
       </c>
-      <c r="C39" s="8" t="inlineStr">
+      <c r="C40" s="8" t="inlineStr">
         <is>
           <t>Valoramos mucho tu privacidad; por ello, te informamos de que el Responsable del tratamiento de datos es SIA "Dynatech". Tus datos personales se utilizarán únicamente para organizar el Quiz del Día Mundial del Turismo y se conservarán durante un período de 30 días.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Result Pages — shared text (applies to all 3 variants)</t>
         </is>
       </c>
-      <c r="B40" s="5" t="n"/>
-      <c r="C40" s="5" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>result.common.label</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Your result</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>Tu resultado</t>
-        </is>
-      </c>
+      <c r="B41" s="5" t="n"/>
+      <c r="C41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>result.common.answers_caption</t>
+          <t>result.common.label</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Correct answers</t>
+          <t>Your result</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Respuestas correctas</t>
+          <t>Tu resultado</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>result.common.time_caption</t>
+          <t>result.common.answers_caption</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Completion time</t>
+          <t>Correct answers</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Tiempo de finalización</t>
+          <t>Respuestas correctas</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>result.common.note_title</t>
+          <t>result.common.time_caption</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>What's next? 🤔</t>
+          <t>Completion time</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>¿Qué sigue? 🤔</t>
+          <t>Tiempo de finalización</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
+          <t>result.common.note_title</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>What's next? 🤔</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>¿Qué sigue? 🤔</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
           <t>result.common.note_description</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="B46" s="7" t="inlineStr">
         <is>
           <t>Thanks for taking part! We've got your scores. Keep an eye on the official Teams channels for the winner announcement. Stay tuned and good luck! ✨</t>
         </is>
       </c>
-      <c r="C45" s="8" t="inlineStr">
+      <c r="C46" s="8" t="inlineStr">
         <is>
           <t>¡Gracias por participar! Ya tenemos tus resultados. Estate atento a los canales oficiales de Teams para el anuncio del ganador. ¡Mantente al tanto y buena suerte! ✨</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>Result Page 1 (1–7 points)</t>
         </is>
       </c>
-      <c r="B46" s="5" t="n"/>
-      <c r="C46" s="5" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>result1.title</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>Curious Tourist</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>Turista Curioso</t>
-        </is>
-      </c>
+      <c r="B47" s="5" t="n"/>
+      <c r="C47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
+          <t>result1.title</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Curious Tourist</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Turista Curioso</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
           <t>result1.description</t>
         </is>
       </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>Every great traveller starts somewhere. Keep exploring, discovering new places, and collecting adventures — next time, you might surprise yourself! ✈️</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="C49" s="8" t="inlineStr">
         <is>
           <t>Todo gran viajero empieza por algún sitio. Sigue explorando, descubriendo nuevos lugares y coleccionando aventuras — ¡la próxima vez podrías sorprenderte a ti mismo! ✈️</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>Result Page 2 (8–12 points)</t>
         </is>
       </c>
-      <c r="B49" s="5" t="n"/>
-      <c r="C49" s="5" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>result2.title</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>World Explorer</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>Explorador del Mundo</t>
-        </is>
-      </c>
+      <c r="B50" s="5" t="n"/>
+      <c r="C50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
+          <t>result2.title</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>World Explorer</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Explorador del Mundo</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
           <t>result2.description</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="B52" s="7" t="inlineStr">
         <is>
           <t>You definitely know your way around the world. Keep traveling, exploring, and discovering — there's always another adventure waiting! 🧭</t>
         </is>
       </c>
-      <c r="C51" s="8" t="inlineStr">
+      <c r="C52" s="8" t="inlineStr">
         <is>
           <t>Definitivamente conoces bien el mundo. Sigue viajando, explorando y descubriendo — ¡siempre hay otra aventura esperando! 🧭</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
         <is>
           <t>Result Page 3 (13–15 points)</t>
         </is>
       </c>
-      <c r="B52" s="5" t="n"/>
-      <c r="C52" s="5" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>result3.title</t>
-        </is>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>Travel Legend</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>Leyenda del Viaje</t>
-        </is>
-      </c>
+      <c r="B53" s="5" t="n"/>
+      <c r="C53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
+          <t>result3.title</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Travel Legend</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>Leyenda del Viaje</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
           <t>result3.description</t>
         </is>
       </c>
-      <c r="B54" s="7" t="inlineStr">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>Wow! Your travel knowledge is impressive. Keep exploring the world and adding even more destinations to your list! 🌎</t>
         </is>
       </c>
-      <c r="C54" s="8" t="inlineStr">
+      <c r="C55" s="8" t="inlineStr">
         <is>
           <t>¡Vaya! Tus conocimientos de viajes son impresionantes. Sigue explorando el mundo y añadiendo aún más destinos a tu lista! 🌎</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>Quiz Questions (1–15) — question text + answer options only</t>
         </is>
       </c>
-      <c r="B55" s="5" t="n"/>
-      <c r="C55" s="5" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t>q1.question</t>
-        </is>
-      </c>
-      <c r="B56" s="7" t="inlineStr">
-        <is>
-          <t>Cartagena, famous for its colourful colonial old town and Caribbean coastline, is located in which country?</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>Cartagena, famosa por su colorida ciudad colonial y su costa caribeña, ¿en qué país se encuentra?</t>
-        </is>
-      </c>
+      <c r="B56" s="5" t="n"/>
+      <c r="C56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>q1.option_a</t>
+          <t>q1.question</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cartagena, famous for its colourful colonial old town and Caribbean coastline, is located in which country?</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cartagena, famosa por su colorida ciudad colonial y su costa caribeña, ¿en qué país se encuentra?</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>q1.option_b</t>
+          <t>q1.option_a</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Venezuela</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Venezuela</t>
+          <t>Colombia</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>q1.option_c</t>
+          <t>q1.option_b</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Venezuela</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>Venezuela</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>q1.option_d</t>
+          <t>q1.option_c</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Panama</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Panamá</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>q2.question</t>
+          <t>q1.option_d</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>What is a “staycation”?</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>¿Qué es una “staycation”?</t>
+          <t>Ecuador</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>q2.option_a</t>
+          <t>q2.question</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>A holiday taken close to or at home</t>
+          <t>What is a “staycation”?</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>Unas vacaciones cerca de casa o en casa</t>
+          <t>¿Qué es una “staycation”?</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>q2.option_b</t>
+          <t>q2.option_a</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>A holiday lasting more than one month</t>
+          <t>A holiday taken close to or at home</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>Unas vacaciones que duran más de un mes</t>
+          <t>Unas vacaciones cerca de casa o en casa</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>q2.option_c</t>
+          <t>q2.option_b</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>A trip involving several overnight flights</t>
+          <t>A holiday lasting more than one month</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>Un viaje que incluye varios vuelos nocturnos</t>
+          <t>Unas vacaciones que duran más de un mes</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>q2.option_d</t>
+          <t>q2.option_c</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>A holiday spent entirely on a cruise ship</t>
+          <t>A trip involving several overnight flights</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>Unas vacaciones que se pasan completamente en un crucero</t>
+          <t>Un viaje que incluye varios vuelos nocturnos</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>q3.question</t>
+          <t>q2.option_d</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Riga, Latvia, is especially well known for having one of Europe's largest collections of which architectural style?</t>
+          <t>A holiday spent entirely on a cruise ship</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Riga, Letonia, es especialmente conocida por tener una de las colecciones más grandes de Europa de edificios de estilo…</t>
+          <t>Unas vacaciones que se pasan completamente en un crucero</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>q3.option_a</t>
+          <t>q3.question</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Baroque</t>
+          <t>Riga, Latvia, is especially well known for having one of Europe's largest collections of which architectural style?</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>Barroco</t>
+          <t>Riga, Letonia, es especialmente conocida por tener una de las colecciones más grandes de Europa de edificios de estilo…</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>q3.option_b</t>
+          <t>q3.option_a</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Art Nouveau</t>
+          <t>Baroque</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>Art Nouveau</t>
+          <t>Barroco</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>q3.option_c</t>
+          <t>q3.option_b</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Gothic Revival</t>
+          <t>Art Nouveau</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>Neogótico</t>
+          <t>Art Nouveau</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>q3.option_d</t>
+          <t>q3.option_c</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Brutalist</t>
+          <t>Gothic Revival</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Brutalista</t>
+          <t>Neogótico</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>q4.question</t>
+          <t>q3.option_d</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>The ancient city of Machu Picchu is one of the most famous tourist attractions in which country?</t>
+          <t>Brutalist</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>La antigua ciudad de Machu Picchu es uno de los atractivos turísticos más famosos de ¿qué país?</t>
+          <t>Brutalista</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>q4.option_a</t>
+          <t>q4.question</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>The ancient city of Machu Picchu is one of the most famous tourist attractions in which country?</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>La antigua ciudad de Machu Picchu es uno de los atractivos turísticos más famosos de ¿qué país?</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>q4.option_b</t>
+          <t>q4.option_a</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>q4.option_c</t>
+          <t>q4.option_b</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>Bolivia</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Bolivia</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>q4.option_d</t>
+          <t>q4.option_c</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Perú</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>q5.question</t>
+          <t>q4.option_d</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>If you want to visit Angkor Wat, which country should you travel to?</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>Si quieres visitar Angkor Wat, ¿a qué país debes viajar?</t>
+          <t>Ecuador</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>q5.option_a</t>
+          <t>q5.question</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>If you want to visit Angkor Wat, which country should you travel to?</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>Tailandia</t>
+          <t>Si quieres visitar Angkor Wat, ¿a qué país debes viajar?</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>q5.option_b</t>
+          <t>q5.option_a</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Tailandia</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>q5.option_c</t>
+          <t>q5.option_b</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>Camboya</t>
+          <t>Vietnam</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>q5.option_d</t>
+          <t>q5.option_c</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Camboya</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>q6.question</t>
+          <t>q5.option_d</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>What does an airport's three-letter code, such as JFK or CDG, usually represent?</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>¿Qué representa normalmente el código de tres letras de un aeropuerto, como JFK o CDG?</t>
+          <t>Indonesia</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>q6.option_a</t>
+          <t>q6.question</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>The airline operating there</t>
+          <t>What does an airport's three-letter code, such as JFK or CDG, usually represent?</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>La aerolínea que opera allí</t>
+          <t>¿Qué representa normalmente el código de tres letras de un aeropuerto, como JFK o CDG?</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>q6.option_b</t>
+          <t>q6.option_a</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>The airport's IATA code</t>
+          <t>The airline operating there</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>El código IATA del aeropuerto</t>
+          <t>La aerolínea que opera allí</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>q6.option_c</t>
+          <t>q6.option_b</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>The runway number</t>
+          <t>The airport's IATA code</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>El número de la pista</t>
+          <t>El código IATA del aeropuerto</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>q6.option_d</t>
+          <t>q6.option_c</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>The country's calling code</t>
+          <t>The runway number</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>El código telefónico del país</t>
+          <t>El número de la pista</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>q7.question</t>
+          <t>q6.option_d</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>The Chocolate Hills, one of the Philippines' most distinctive natural attractions, are located on which island?</t>
+          <t>The country's calling code</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>Las Chocolate Hills, uno de los atractivos naturales más característicos de Filipinas, ¿en qué isla se encuentran?</t>
+          <t>El código telefónico del país</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>q7.option_a</t>
+          <t>q7.question</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>Palawan</t>
+          <t>The Chocolate Hills, one of the Philippines' most distinctive natural attractions, are located on which island?</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>Palawan</t>
+          <t>Las Chocolate Hills, uno de los atractivos naturales más característicos de Filipinas, ¿en qué isla se encuentran?</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>q7.option_b</t>
+          <t>q7.option_a</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>Bohol</t>
+          <t>Palawan</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>Bohol</t>
+          <t>Palawan</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>q7.option_c</t>
+          <t>q7.option_b</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>Cebu</t>
+          <t>Bohol</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>Cebú</t>
+          <t>Bohol</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>q7.option_d</t>
+          <t>q7.option_c</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>Luzon</t>
+          <t>Cebu</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>Luzón</t>
+          <t>Cebú</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>q8.question</t>
+          <t>q7.option_d</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>Which high-speed train service connects major cities such as Paris, Brussels, Amsterdam and Cologne?</t>
+          <t>Luzon</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>¿Qué servicio de tren de alta velocidad conecta importantes ciudades como París, Bruselas, Ámsterdam y Colonia?</t>
+          <t>Luzón</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>q8.option_a</t>
+          <t>q8.question</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>Eurostar</t>
+          <t>Which high-speed train service connects major cities such as Paris, Brussels, Amsterdam and Cologne?</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>Eurostar</t>
+          <t>¿Qué servicio de tren de alta velocidad conecta importantes ciudades como París, Bruselas, Ámsterdam y Colonia?</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>q8.option_b</t>
+          <t>q8.option_a</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>Thalys</t>
+          <t>Eurostar</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>Thalys</t>
+          <t>Eurostar</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>q8.option_c</t>
+          <t>q8.option_b</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>Glacier Express</t>
+          <t>Thalys</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t>Glacier Express</t>
+          <t>Thalys</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>q8.option_d</t>
+          <t>q8.option_c</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>Orient Express</t>
+          <t>Glacier Express</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t>Orient Express</t>
+          <t>Glacier Express</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>q9.question</t>
+          <t>q8.option_d</t>
         </is>
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>Which famous landmark would you visit in Agra, India?</t>
+          <t>Orient Express</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t>¿Qué famoso lugar emblemático visitarías en Agra, India?</t>
+          <t>Orient Express</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>q9.option_a</t>
+          <t>q9.question</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>Golden Temple</t>
+          <t>Which famous landmark would you visit in Agra, India?</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>Templo Dorado</t>
+          <t>¿Qué famoso lugar emblemático visitarías en Agra, India?</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>q9.option_b</t>
+          <t>q9.option_a</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t>Taj Mahal</t>
+          <t>Golden Temple</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t>Taj Mahal</t>
+          <t>Templo Dorado</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>q9.option_c</t>
+          <t>q9.option_b</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>Gateway of India</t>
+          <t>Taj Mahal</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t>Puerta de la India</t>
+          <t>Taj Mahal</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>q9.option_d</t>
+          <t>q9.option_c</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
         <is>
-          <t>Lotus Temple</t>
+          <t>Gateway of India</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t>Templo del Loto</t>
+          <t>Puerta de la India</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>q10.question</t>
+          <t>q9.option_d</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
         <is>
-          <t>Which major European airport is located partly below sea level?</t>
+          <t>Lotus Temple</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t>¿Cuál de estos importantes aeropuertos europeos está ubicado parcialmente por debajo del nivel del mar?</t>
+          <t>Templo del Loto</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>q10.option_a</t>
+          <t>q10.question</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
         <is>
-          <t>Frankfurt Airport</t>
+          <t>Which major European airport is located partly below sea level?</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>Aeropuerto de Frankfurt</t>
+          <t>¿Cuál de estos importantes aeropuertos europeos está ubicado parcialmente por debajo del nivel del mar?</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>q10.option_b</t>
+          <t>q10.option_a</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
         <is>
-          <t>Amsterdam Schiphol Airport</t>
+          <t>Frankfurt Airport</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>Aeropuerto de Ámsterdam-Schiphol</t>
+          <t>Aeropuerto de Frankfurt</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>q10.option_c</t>
+          <t>q10.option_b</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
         <is>
-          <t>Madrid Barajas Airport</t>
+          <t>Amsterdam Schiphol Airport</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t>Aeropuerto Adolfo Suárez Madrid-Barajas</t>
+          <t>Aeropuerto de Ámsterdam-Schiphol</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>q10.option_d</t>
+          <t>q10.option_c</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
-          <t>Zurich Airport</t>
+          <t>Madrid Barajas Airport</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t>Aeropuerto de Zúrich</t>
+          <t>Aeropuerto Adolfo Suárez Madrid-Barajas</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>q11.question</t>
+          <t>q10.option_d</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>The spectacular Registan Square, surrounded by three historic madrasas, is one of the best-known attractions in which Uzbek city?</t>
+          <t>Zurich Airport</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t>La espectacular Plaza Registán, rodeada por tres madrasas históricas, es uno de los atractivos más conocidos de ¿qué ciudad de Uzbekistán?</t>
+          <t>Aeropuerto de Zúrich</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>q11.option_a</t>
+          <t>q11.question</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
         <is>
-          <t>Tashkent</t>
+          <t>The spectacular Registan Square, surrounded by three historic madrasas, is one of the best-known attractions in which Uzbek city?</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t>Taskent</t>
+          <t>La espectacular Plaza Registán, rodeada por tres madrasas históricas, es uno de los atractivos más conocidos de ¿qué ciudad de Uzbekistán?</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>q11.option_b</t>
+          <t>q11.option_a</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>Bukhara</t>
+          <t>Tashkent</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t>Bujará</t>
+          <t>Taskent</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>q11.option_c</t>
+          <t>q11.option_b</t>
         </is>
       </c>
       <c r="B109" s="7" t="inlineStr">
         <is>
-          <t>Samarkand</t>
+          <t>Bukhara</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t>Samarcanda</t>
+          <t>Bujará</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>q11.option_d</t>
+          <t>q11.option_c</t>
         </is>
       </c>
       <c r="B110" s="7" t="inlineStr">
         <is>
-          <t>Khiva</t>
+          <t>Samarkand</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t>Jiva</t>
+          <t>Samarcanda</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>q12.question</t>
+          <t>q11.option_d</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>Which city welcomed the most international visitors in the world in 2025?</t>
+          <t>Khiva</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t>¿Qué ciudad recibió la mayor cantidad de visitantes internacionales del mundo en 2025?</t>
+          <t>Jiva</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>q12.option_a</t>
+          <t>q12.question</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Which city welcomed the most international visitors in the world in 2025?</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t>París</t>
+          <t>¿Qué ciudad recibió la mayor cantidad de visitantes internacionales del mundo en 2025?</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>q12.option_b</t>
+          <t>q12.option_a</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t>Londres</t>
+          <t>París</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>q12.option_c</t>
+          <t>q12.option_b</t>
         </is>
       </c>
       <c r="B114" s="7" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>London</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Londres</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>q12.option_d</t>
+          <t>q12.option_c</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Bangkok</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t>Dubái</t>
+          <t>Bangkok</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>q13.question</t>
+          <t>q12.option_d</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
         <is>
-          <t>Chișinău is Moldova's capital, but which river runs through the city?</t>
+          <t>Dubai</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t>Chișinău es la capital de Moldavia, pero ¿qué río atraviesa la ciudad?</t>
+          <t>Dubái</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>q13.option_a</t>
+          <t>q13.question</t>
         </is>
       </c>
       <c r="B117" s="7" t="inlineStr">
         <is>
-          <t>Dniester</t>
+          <t>Chișinău is Moldova's capital, but which river runs through the city?</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t>Dniéster</t>
+          <t>Chișinău es la capital de Moldavia, pero ¿qué río atraviesa la ciudad?</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>q13.option_b</t>
+          <t>q13.option_a</t>
         </is>
       </c>
       <c r="B118" s="7" t="inlineStr">
         <is>
-          <t>Prut</t>
+          <t>Dniester</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t>Prut</t>
+          <t>Dniéster</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>q13.option_c</t>
+          <t>q13.option_b</t>
         </is>
       </c>
       <c r="B119" s="7" t="inlineStr">
         <is>
-          <t>Bîc</t>
+          <t>Prut</t>
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t>Bîc</t>
+          <t>Prut</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>q13.option_d</t>
+          <t>q13.option_c</t>
         </is>
       </c>
       <c r="B120" s="7" t="inlineStr">
         <is>
-          <t>Danube</t>
+          <t>Bîc</t>
         </is>
       </c>
       <c r="C120" s="8" t="inlineStr">
         <is>
-          <t>Danubio</t>
+          <t>Bîc</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>q14.question</t>
+          <t>q13.option_d</t>
         </is>
       </c>
       <c r="B121" s="7" t="inlineStr">
         <is>
-          <t>Which famous landmark is often described as the most visited paid monument in the world?</t>
+          <t>Danube</t>
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr">
         <is>
-          <t>¿Qué famoso lugar emblemático suele ser descrito como el monumento de pago más visitado del mundo?</t>
+          <t>Danubio</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>q14.option_a</t>
+          <t>q14.question</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
         <is>
-          <t>Taj Mahal</t>
+          <t>Which famous landmark is often described as the most visited paid monument in the world?</t>
         </is>
       </c>
       <c r="C122" s="8" t="inlineStr">
         <is>
-          <t>Taj Mahal</t>
+          <t>¿Qué famoso lugar emblemático suele ser descrito como el monumento de pago más visitado del mundo?</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>q14.option_b</t>
+          <t>q14.option_a</t>
         </is>
       </c>
       <c r="B123" s="7" t="inlineStr">
         <is>
-          <t>Eiffel Tower</t>
+          <t>Taj Mahal</t>
         </is>
       </c>
       <c r="C123" s="8" t="inlineStr">
         <is>
-          <t>Torre Eiffel</t>
+          <t>Taj Mahal</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>q14.option_c</t>
+          <t>q14.option_b</t>
         </is>
       </c>
       <c r="B124" s="7" t="inlineStr">
         <is>
-          <t>Colosseum</t>
+          <t>Eiffel Tower</t>
         </is>
       </c>
       <c r="C124" s="8" t="inlineStr">
         <is>
-          <t>Coliseo</t>
+          <t>Torre Eiffel</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>q14.option_d</t>
+          <t>q14.option_c</t>
         </is>
       </c>
       <c r="B125" s="7" t="inlineStr">
         <is>
-          <t>Empire State Building</t>
+          <t>Colosseum</t>
         </is>
       </c>
       <c r="C125" s="8" t="inlineStr">
         <is>
-          <t>Empire State Building</t>
+          <t>Coliseo</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>q15.question</t>
+          <t>q14.option_d</t>
         </is>
       </c>
       <c r="B126" s="7" t="inlineStr">
         <is>
-          <t>Final challenge: Match the famous attraction with the correct city. Which combination is WRONG?</t>
+          <t>Empire State Building</t>
         </is>
       </c>
       <c r="C126" s="8" t="inlineStr">
         <is>
-          <t>Desafío final: relaciona cada atracción famosa con la ciudad correcta. ¿Cuál de estas combinaciones es INCORRECTA?</t>
+          <t>Empire State Building</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>q15.option_a</t>
+          <t>q15.question</t>
         </is>
       </c>
       <c r="B127" s="7" t="inlineStr">
         <is>
-          <t>Trevi Fountain – Rome</t>
+          <t>Final challenge: Match the famous attraction with the correct city. Which combination is WRONG?</t>
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr">
         <is>
-          <t>Fontana di Trevi – Roma</t>
+          <t>Desafío final: relaciona cada atracción famosa con la ciudad correcta. ¿Cuál de estas combinaciones es INCORRECTA?</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>q15.option_b</t>
+          <t>q15.option_a</t>
         </is>
       </c>
       <c r="B128" s="7" t="inlineStr">
         <is>
-          <t>Acropolis – Athens</t>
+          <t>Trevi Fountain – Rome</t>
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr">
         <is>
-          <t>Acrópolis – Atenas</t>
+          <t>Fontana di Trevi – Roma</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>q15.option_c</t>
+          <t>q15.option_b</t>
         </is>
       </c>
       <c r="B129" s="7" t="inlineStr">
         <is>
-          <t>Golden Gate Bridge – Los Angeles</t>
+          <t>Acropolis – Athens</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
         <is>
-          <t>Golden Gate Bridge – Los Ángeles</t>
+          <t>Acrópolis – Atenas</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
         <is>
+          <t>q15.option_c</t>
+        </is>
+      </c>
+      <c r="B130" s="7" t="inlineStr">
+        <is>
+          <t>Golden Gate Bridge – Los Angeles</t>
+        </is>
+      </c>
+      <c r="C130" s="8" t="inlineStr">
+        <is>
+          <t>Golden Gate Bridge – Los Ángeles</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="6" t="inlineStr">
+        <is>
           <t>q15.option_d</t>
         </is>
       </c>
-      <c r="B130" s="7" t="inlineStr">
+      <c r="B131" s="7" t="inlineStr">
         <is>
           <t>Marina Bay Sands – Singapore</t>
         </is>
       </c>
-      <c r="C130" s="8" t="inlineStr">
+      <c r="C131" s="8" t="inlineStr">
         <is>
           <t>Marina Bay Sands – Singapur</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="4" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="4" t="inlineStr">
         <is>
           <t>Quiz Question — Submit Button (default state)</t>
         </is>
       </c>
-      <c r="B131" s="5" t="n"/>
-      <c r="C131" s="5" t="n"/>
-    </row>
-    <row r="132">
-      <c r="A132" s="6" t="inlineStr">
+      <c r="B132" s="5" t="n"/>
+      <c r="C132" s="5" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="6" t="inlineStr">
         <is>
           <t>quiz.submit_button_default</t>
         </is>
       </c>
-      <c r="B132" s="7" t="inlineStr">
+      <c r="B133" s="7" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="C132" s="8" t="inlineStr">
+      <c r="C133" s="8" t="inlineStr">
         <is>
           <t>Enviar</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" s="4" t="inlineStr">
+    <row r="134">
+      <c r="A134" s="4" t="inlineStr">
         <is>
           <t>Answer Feedback Messages (shown on the Submit button after answering)</t>
         </is>
       </c>
-      <c r="B133" s="5" t="n"/>
-      <c r="C133" s="5" t="n"/>
-    </row>
-    <row r="134">
-      <c r="A134" s="6" t="inlineStr">
-        <is>
-          <t>feedback.correct.1</t>
-        </is>
-      </c>
-      <c r="B134" s="7" t="inlineStr">
-        <is>
-          <t>Correct! 🥳</t>
-        </is>
-      </c>
-      <c r="C134" s="8" t="inlineStr">
-        <is>
-          <t>¡Correcto! 🥳</t>
-        </is>
-      </c>
+      <c r="B134" s="5" t="n"/>
+      <c r="C134" s="5" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>feedback.correct.2</t>
+          <t>feedback.correct.1</t>
         </is>
       </c>
       <c r="B135" s="7" t="inlineStr">
         <is>
-          <t>Just wow! 👏</t>
+          <t>Correct! 🥳</t>
         </is>
       </c>
       <c r="C135" s="8" t="inlineStr">
         <is>
-          <t>¡Vaya! 👏</t>
+          <t>¡Correcto! 🥳</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>feedback.correct.3</t>
+          <t>feedback.correct.2</t>
         </is>
       </c>
       <c r="B136" s="7" t="inlineStr">
         <is>
-          <t>Amazing! 🤩</t>
+          <t>Just wow! 👏</t>
         </is>
       </c>
       <c r="C136" s="8" t="inlineStr">
         <is>
-          <t>¡Increíble! 🤩</t>
+          <t>¡Vaya! 👏</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>feedback.correct.4</t>
+          <t>feedback.correct.3</t>
         </is>
       </c>
       <c r="B137" s="7" t="inlineStr">
         <is>
-          <t>Nailed it! 💅</t>
+          <t>Amazing! 🤩</t>
         </is>
       </c>
       <c r="C137" s="8" t="inlineStr">
         <is>
-          <t>¡Acertaste! 💅</t>
+          <t>¡Increíble! 🤩</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>feedback.correct.5</t>
+          <t>feedback.correct.4</t>
         </is>
       </c>
       <c r="B138" s="7" t="inlineStr">
         <is>
-          <t>You are on fire! 💃</t>
+          <t>Nailed it! 💅</t>
         </is>
       </c>
       <c r="C138" s="8" t="inlineStr">
         <is>
-          <t>¡Estás que ardes! 💃</t>
+          <t>¡Acertaste! 💅</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>feedback.wrong.1</t>
+          <t>feedback.correct.5</t>
         </is>
       </c>
       <c r="B139" s="7" t="inlineStr">
         <is>
-          <t>Now you know... 🤷🏻‍♀️</t>
+          <t>You are on fire! 💃</t>
         </is>
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t>Ahora ya lo sabes... 🤷🏻‍♀️</t>
+          <t>¡Estás que ardes! 💃</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>feedback.wrong.2</t>
+          <t>feedback.wrong.1</t>
         </is>
       </c>
       <c r="B140" s="7" t="inlineStr">
         <is>
-          <t>So close! 👀</t>
+          <t>Now you know... 🤷🏻‍♀️</t>
         </is>
       </c>
       <c r="C140" s="8" t="inlineStr">
         <is>
-          <t>¡Tan cerca! 👀</t>
+          <t>Ahora ya lo sabes... 🤷🏻‍♀️</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>feedback.wrong.3</t>
+          <t>feedback.wrong.2</t>
         </is>
       </c>
       <c r="B141" s="7" t="inlineStr">
         <is>
-          <t>We're always learning 🧐</t>
+          <t>So close! 👀</t>
         </is>
       </c>
       <c r="C141" s="8" t="inlineStr">
         <is>
-          <t>Siempre se aprende 🧐</t>
+          <t>¡Tan cerca! 👀</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>feedback.wrong.4</t>
+          <t>feedback.wrong.3</t>
         </is>
       </c>
       <c r="B142" s="7" t="inlineStr">
         <is>
-          <t>Hmmm 🤔</t>
+          <t>We're always learning 🧐</t>
         </is>
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t>Hmmm 🤔</t>
+          <t>Siempre se aprende 🧐</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
+          <t>feedback.wrong.4</t>
+        </is>
+      </c>
+      <c r="B143" s="7" t="inlineStr">
+        <is>
+          <t>Hmmm 🤔</t>
+        </is>
+      </c>
+      <c r="C143" s="8" t="inlineStr">
+        <is>
+          <t>Hmmm 🤔</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="6" t="inlineStr">
+        <is>
           <t>feedback.wrong.5</t>
         </is>
       </c>
-      <c r="B143" s="7" t="inlineStr">
+      <c r="B144" s="7" t="inlineStr">
         <is>
           <t>Oops 🙈</t>
         </is>
       </c>
-      <c r="C143" s="8" t="inlineStr">
+      <c r="C144" s="8" t="inlineStr">
         <is>
           <t>Ups 🙈</t>
         </is>

</xml_diff>